<commit_message>
sprint 1 self assessment file correction
</commit_message>
<xml_diff>
--- a/scrum/SEM3-PI2526-SA-G091-Sprint1.xlsx
+++ b/scrum/SEM3-PI2526-SA-G091-Sprint1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joaom\OneDrive\Ambiente de Trabalho\Licenciatura\LEI - 2ºano\1º Semestre\Projeto Integrador\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9e9f88227fd1257f/Ambiente de Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E1F2C55-E43F-4159-9A9E-C3D2ABB8E3A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A9AA365-AE70-42AC-9246-78DF660831D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-180" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Team and Self Assessment" sheetId="2" r:id="rId1"/>
@@ -1380,33 +1380,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:I28"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="6.25" customWidth="1"/>
-    <col min="3" max="3" width="13.25" customWidth="1"/>
-    <col min="4" max="8" width="7.875" customWidth="1"/>
+    <col min="2" max="2" width="6.19921875" customWidth="1"/>
+    <col min="3" max="3" width="13.19921875" customWidth="1"/>
+    <col min="4" max="8" width="7.8984375" customWidth="1"/>
     <col min="9" max="9" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
         <v>37</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
         <v>35</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>0</v>
       </c>
@@ -1415,13 +1415,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:9" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:9" ht="15.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="E8" s="53" t="s">
@@ -1432,7 +1432,7 @@
       <c r="H8" s="54"/>
       <c r="I8" s="55"/>
     </row>
-    <row r="9" spans="1:9" ht="105.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="105.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="27" t="str">
@@ -1455,7 +1455,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="51" t="s">
         <v>5</v>
       </c>
@@ -1479,49 +1479,73 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="52"/>
       <c r="C11" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="49"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="33" t="e">
+      <c r="D11" s="7">
+        <v>4</v>
+      </c>
+      <c r="E11" s="49">
+        <v>4</v>
+      </c>
+      <c r="F11" s="23">
+        <v>4</v>
+      </c>
+      <c r="G11" s="6">
+        <v>4</v>
+      </c>
+      <c r="H11" s="33">
         <f>AVERAGE(D11:G11)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="52"/>
       <c r="C12" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="49"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="33" t="e">
+      <c r="D12" s="6">
+        <v>4</v>
+      </c>
+      <c r="E12" s="7">
+        <v>4</v>
+      </c>
+      <c r="F12" s="49">
+        <v>4</v>
+      </c>
+      <c r="G12" s="23">
+        <v>4</v>
+      </c>
+      <c r="H12" s="33">
         <f>AVERAGE(D12:G12)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="46.5" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="30.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="52"/>
       <c r="C13" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="49"/>
-      <c r="H13" s="33" t="e">
+      <c r="D13" s="6">
+        <v>4</v>
+      </c>
+      <c r="E13" s="6">
+        <v>4</v>
+      </c>
+      <c r="F13" s="7">
+        <v>4</v>
+      </c>
+      <c r="G13" s="49">
+        <v>4</v>
+      </c>
+      <c r="H13" s="33">
         <f>AVERAGE(D13:G13)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="31.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="31.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="1"/>
       <c r="C14" s="30" t="s">
         <v>36</v>
@@ -1544,7 +1568,7 @@
       </c>
       <c r="H14" s="34"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="38" t="s">
         <v>6</v>
       </c>
@@ -1556,7 +1580,7 @@
       <c r="G16" s="39"/>
       <c r="H16" s="40"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="41" t="s">
         <v>34</v>
       </c>
@@ -1568,7 +1592,7 @@
       <c r="G17" s="42"/>
       <c r="H17" s="43"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="44" t="s">
         <v>31</v>
       </c>
@@ -1580,7 +1604,7 @@
       <c r="G18" s="42"/>
       <c r="H18" s="43"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="50" t="s">
         <v>38</v>
       </c>
@@ -1592,7 +1616,7 @@
       <c r="G19" s="42"/>
       <c r="H19" s="43"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="41"/>
       <c r="B20" s="42"/>
       <c r="C20" s="42"/>
@@ -1602,7 +1626,7 @@
       <c r="G20" s="42"/>
       <c r="H20" s="43"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="45" t="s">
         <v>32</v>
       </c>
@@ -1614,7 +1638,7 @@
       <c r="G21" s="42"/>
       <c r="H21" s="43"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="41">
         <v>0</v>
       </c>
@@ -1628,7 +1652,7 @@
       <c r="G22" s="42"/>
       <c r="H22" s="43"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="41">
         <v>1</v>
       </c>
@@ -1642,7 +1666,7 @@
       <c r="G23" s="42"/>
       <c r="H23" s="43"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="41">
         <v>2</v>
       </c>
@@ -1656,7 +1680,7 @@
       <c r="G24" s="42"/>
       <c r="H24" s="43"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="41">
         <v>3</v>
       </c>
@@ -1670,7 +1694,7 @@
       <c r="G25" s="42"/>
       <c r="H25" s="43"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="41">
         <v>4</v>
       </c>
@@ -1684,7 +1708,7 @@
       <c r="G26" s="42"/>
       <c r="H26" s="43"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="41">
         <v>5</v>
       </c>
@@ -1698,7 +1722,7 @@
       <c r="G27" s="42"/>
       <c r="H27" s="43"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="46"/>
       <c r="B28" s="47"/>
       <c r="C28" s="47"/>
@@ -1727,7 +1751,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="20.125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="20.09765625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5" customWidth="1"/>
     <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
@@ -1735,13 +1759,13 @@
     <col min="5" max="10" width="27.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="18" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="51" t="s">
         <v>14</v>
       </c>
@@ -1773,7 +1797,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A4" s="52"/>
       <c r="B4" s="59"/>
       <c r="C4" s="59"/>
@@ -1797,7 +1821,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="52"/>
       <c r="B5" s="59"/>
       <c r="C5" s="59"/>
@@ -1821,7 +1845,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A6" s="10"/>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
@@ -1845,7 +1869,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A7" s="10"/>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
@@ -1869,7 +1893,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A8" s="10"/>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -1893,7 +1917,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A9" s="10"/>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -1917,7 +1941,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A10" s="10"/>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
@@ -1941,7 +1965,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A11" s="10"/>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
@@ -1965,7 +1989,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A12" s="10"/>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
@@ -1989,7 +2013,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A13" s="10"/>
       <c r="B13" s="17"/>
       <c r="C13" s="17"/>
@@ -2013,7 +2037,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A14" s="10"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
@@ -2037,7 +2061,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A15" s="10"/>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -2061,7 +2085,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A16" s="10"/>
       <c r="B16" s="17"/>
       <c r="C16" s="17"/>
@@ -2085,7 +2109,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
@@ -2109,7 +2133,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A18" s="10"/>
       <c r="B18" s="17"/>
       <c r="C18" s="17"/>
@@ -2133,7 +2157,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A19" s="10"/>
       <c r="B19" s="17"/>
       <c r="C19" s="17"/>
@@ -2157,7 +2181,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A20" s="10"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -2181,7 +2205,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A21" s="10"/>
       <c r="B21" s="17"/>
       <c r="C21" s="17"/>
@@ -2205,7 +2229,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A22" s="10"/>
       <c r="B22" s="17"/>
       <c r="C22" s="17"/>
@@ -2229,7 +2253,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A23" s="10"/>
       <c r="B23" s="17"/>
       <c r="C23" s="17"/>
@@ -2253,7 +2277,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
       <c r="B24" s="17"/>
       <c r="C24" s="17"/>
@@ -2277,7 +2301,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A25" s="10"/>
       <c r="B25" s="17"/>
       <c r="C25" s="17"/>
@@ -2301,7 +2325,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A26" s="10"/>
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
@@ -2325,7 +2349,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A27" s="10"/>
       <c r="B27" s="17"/>
       <c r="C27" s="17"/>
@@ -2349,7 +2373,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A28" s="10"/>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
@@ -2373,7 +2397,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A29" s="10"/>
       <c r="B29" s="17"/>
       <c r="C29" s="17"/>
@@ -2397,7 +2421,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
         <v>33</v>
       </c>
@@ -2423,7 +2447,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
       <c r="B31" s="17"/>
       <c r="C31" s="17"/>
@@ -2447,7 +2471,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="48" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="14"/>
       <c r="B32" s="35"/>
       <c r="C32" s="17"/>
@@ -2514,6 +2538,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005836243B3C47804EAF5FFDD9F066FCC7" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d21ddf3f0b128e39c9d770c8c903166">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0326308c339679ad994635f2c691325" ns2:_="">
     <xsd:import namespace="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
@@ -2697,12 +2727,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
   <ds:schemaRefs>
@@ -2712,6 +2736,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B77F7C-EE47-4FBD-B078-6536C1487A1E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2727,20 +2767,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>